<commit_message>
Update inventory import file
</commit_message>
<xml_diff>
--- a/imports/import_inventory_ONE_SHEET_PER_PRODUCT.xlsx
+++ b/imports/import_inventory_ONE_SHEET_PER_PRODUCT.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D117BEF-85C5-4BEB-B6E5-67B4072AF137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0494499B-EE98-40E2-B25D-E99E5407437C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GEMINI" sheetId="1" r:id="rId1"/>
-    <sheet name="CAPCUT" sheetId="2" r:id="rId2"/>
+    <sheet name="CHAT GPT" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
   <si>
     <t>product_code</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>30D</t>
-  </si>
-  <si>
-    <t>sanylionmeyakhalifa@gmail.com|Siam@1122|hylz h4io nbdc ukqf lueo hvse souu 3rnn</t>
   </si>
   <si>
     <t>GOOGLE AI PRO (GEMINI) – 1 THÁNG
@@ -93,38 +90,57 @@
     <t>dmajijur70@gmail.com|Siam@1122|2FA: 25uw cbyn shz4 ebi5 hazk kfev ut7y 67ol</t>
   </si>
   <si>
-    <t>mdabirkhanyz@gmail.com|Siam@1122|2FA: 25uw cbyn shz4 ebi5 hazk kfev ut7y 67o</t>
-  </si>
-  <si>
-    <t>mdabirxxzzcc11@gmail.com|Siam@1122|2FA: ap5w vmlg sdms 34oz wqs5 4act jwzy 5m22</t>
-  </si>
-  <si>
-    <t>CAPCUT</t>
-  </si>
-  <si>
-    <t>CAPCUT PRO</t>
-  </si>
-  <si>
-    <t>365D</t>
-  </si>
-  <si>
-    <t>phamanhduong5599@gmail.com|79Gml5599@</t>
-  </si>
-  <si>
-    <t>CapCut Pro 1 năm - tài khoản cá nhân. Đăng nhập bằng email và mật khẩu được cung cấp.</t>
-  </si>
-  <si>
-    <t>phamanhduong6699@gmail.com|79Gml5599@</t>
-  </si>
-  <si>
-    <t>phamanhduong7799@gmail.com|79Gml5599@</t>
+    <t>CHAT GPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Plus - 1 THÁNG</t>
+  </si>
+  <si>
+    <t>chaturangaant@gmail.com|Fi5k3fi57cx#|B4N2SE3ENOGSQUARF3S3RNUXGLJP2FMV</t>
+  </si>
+  <si>
+    <t>• Được đảm bảo trạng thái GPT Plus ngay khi đăng nhập lần đầu.
+• Tài khoản cá nhân chất lượng cao, sẵn sàng sử dụng ngay lập tức.
+• Giao hàng nhanh chóng và an toàn sau khi mua hàng
+» Bảo hành: Chúng tôi cung cấp bảo hành 72 giờ sau khi giao hàng thành công. Trong thời gian này, chúng tôi sẽ hỗ trợ đổi trả nếu tài khoản gặp sự cố đăng nhập hoặc không có trạng thái GPT Plus khi đăng nhập lần đầu. Bảo hành này không bao gồm các vấn đề liên quan đến Codex, giới hạn sử dụng, hạn chế hoặc bất kỳ vấn đề nào do chính sách của OpenAI gây ra.
+➤ Thông tin mới
+Đây là tài khoản Plus dùng thử. Mặc dù bạn sẽ nhận được quyền truy cập GPT Plus ngay khi đăng nhập lần đầu, nhưng OpenAI gần đây đã siết chặt hơn việc giám sát sử dụng. Việc sử dụng quá nhiều, số lượng thông báo nhanh chóng hoặc các kiểu hoạt động bất thường có thể dẫn đến việc hạn chế tài khoản tạm thời hoặc vĩnh viễn.
+Nếu bạn gặp bất kỳ giới hạn sử dụng, tốc độ chậm hoặc sự cố truy cập nào, vui lòng hiểu rằng điều này là do chính sách thắt chặt của OpenAI đối với tài khoản Plus. Chúng tôi cung cấp giải pháp này trong thời gian ngắn và không thể đảm bảo tính ổn định trong suốt một tháng khi sử dụng nhiều.
+➤ 𝐀𝐛𝐨𝐮𝐭 𝐏𝐡𝐨𝐧𝐞 𝐍𝐮𝐦𝐛𝐞𝐫 𝐟𝐨𝐫 𝐂𝐨𝐝𝐞𝐱 𝐂𝐨𝐧𝐧𝐞𝐜𝐭𝐢𝐨𝐧
+Chúng tôi có thể cung cấp số điện thoại dùng một lần nếu cần. Tuy nhiên, chúng tôi đặc biệt khuyến nghị bạn sử dụng số WhatsApp hoặc số điện thoại cá nhân của mình để xác minh. Số điện thoại dùng một lần không thể sử dụng lại nếu Codex yêu cầu mã xác minh lần nữa sau này.
+Nếu bạn vẫn cần mã số sử dụng một lần, vui lòng liên hệ với chúng tôi ngay sau khi mua hàng.
+➤ 𝐇𝐨𝐰 𝐭𝐨 𝐋𝐨𝐠 𝐈𝐧 (𝐒𝐮𝐩𝐞𝐫 𝐄𝐚𝐬𝐲)
+Sau khi mua hàng, bạn sẽ nhận được:
+Email • Mật khẩu • Mã TOTP (Mã bí mật xác thực hai yếu tố)
+Hướng dẫn từng bước:
+1. Nhập Email và Mật khẩu.
+2. Khi được yêu cầu nhập mã xác minh 6 chữ số, hãy truy cập 2fa.live.
+3. Dán mã TOTP (mã bí mật xác thực hai yếu tố) mà chúng tôi đã cung cấp (Ví dụ: HOYQ6HSFSRSGUWS2YIQFHJYGHIC66G2G) → Nhấn "Lấy mã".
+4. Sao chép mã 6 chữ số được tạo ra và dán vào OpenAI / GPT.
+Lưu ý quan trọng: Nếu bạn gặp lỗi hoặc không thấy các bước hướng dẫn, vui lòng xóa bộ nhớ cache của trình duyệt, thử đăng nhập lại trên tab mới hoặc sử dụng trình duyệt khác.
+⚡ Giao hàng tức thì | Truy cập toàn cầu
+Bao gồm:
+- Gemini Advanced
+- 1.000 Google Flow Credits / tháng
+- NotebookLM Pro
+- Google Flow AI Creative Studio
+- Google One 5TB
+- Gmail, Docs, Sheets
+Đăng nhập:
+- Email + Password
+- Thêm mã Google Authenticator (2FA)
+Lưu ý:
+- Không thay đổi thông tin đăng nhập hoặc cài đặt bảo mật trong 7 ngày đầu.
+- Một số tính năng có thể kích hoạt sau 3–7 ngày.
+Thời hạn sử dụng: 1 tháng
+Bảo hành: 1 tháng.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -133,6 +149,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -158,10 +180,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -177,8 +200,12 @@
         </x:ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -212,7 +239,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="GEMINITable" displayName="GEMINITable" ref="A1:J9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="GEMINITable" displayName="GEMINITable" ref="A1:J2">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="product_code"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="category"/>
@@ -230,18 +257,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="CAPCUTTable" displayName="CAPCUTTable" ref="A1:J4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{89253D10-2CDF-479E-9130-ED2A22F2316A}" name="GEMINITable4" displayName="GEMINITable4" ref="A1:J2">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="product_code"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="category"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="product_name"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="account_type"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="duration"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="price_vnd"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="warranty_days"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="credential_text"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="note"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="active"/>
+    <tableColumn id="1" xr3:uid="{AA6210DF-5134-4077-9E3F-4A7115D828F1}" name="product_code"/>
+    <tableColumn id="2" xr3:uid="{4F8A6971-2D81-40DD-8517-FF0F4B212BA0}" name="category"/>
+    <tableColumn id="3" xr3:uid="{1D9BC01F-7C61-410B-B12A-4D748F08AD42}" name="product_name"/>
+    <tableColumn id="4" xr3:uid="{9EA9F053-285B-49A2-8C79-F17660BA2ECC}" name="account_type"/>
+    <tableColumn id="5" xr3:uid="{F01358CF-FE37-4A13-A9C7-E46D39AC999F}" name="duration"/>
+    <tableColumn id="6" xr3:uid="{077FFA1C-75CB-4D85-AC76-7690A5608820}" name="price_vnd"/>
+    <tableColumn id="7" xr3:uid="{AC85F74D-F3AC-45C8-9185-91268F84FF71}" name="warranty_days"/>
+    <tableColumn id="8" xr3:uid="{5427A69D-FA0F-4BED-9D86-4485C72AFE33}" name="credential_text"/>
+    <tableColumn id="9" xr3:uid="{860E2184-BE9D-4A51-9033-5BD8CDF96DD8}" name="note"/>
+    <tableColumn id="10" xr3:uid="{65781652-88E4-4014-88AD-A921FFB342BE}" name="active"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -396,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -465,236 +492,12 @@
         <v>30</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="J2" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="33" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G3" s="2">
-        <v>30</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="33" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G4" s="2">
-        <v>30</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="33" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G5" s="2">
-        <v>30</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="33" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G6" s="2">
-        <v>30</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="33" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G7" s="2">
-        <v>30</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="33" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G8" s="2">
-        <v>30</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="33" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="2">
-        <v>70000</v>
-      </c>
-      <c r="G9" s="2">
-        <v>30</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -707,8 +510,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688296D8-B261-4A05-A996-60F412925360}">
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -754,106 +557,45 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="72" customHeight="1">
+    <row r="2" spans="1:10" ht="33" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F2" s="2">
-        <v>400000</v>
+        <v>160000</v>
       </c>
       <c r="G2" s="2">
-        <v>365</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J2" s="3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="72" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="2">
-        <v>400000</v>
-      </c>
-      <c r="G3" s="2">
-        <v>365</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="72" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="2">
-        <v>400000</v>
-      </c>
-      <c r="G4" s="2">
-        <v>365</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" s="3" t="b">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{F5169B72-8ACF-4A67-9963-7EC039AFF531}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>